<commit_message>
Simplificar evidencias y flujo operativo del curso
</commit_message>
<xml_diff>
--- a/02-PROFESORADO/05-ECOSISTEMA-DIGITAL/PLANTILLAS-MAESTRAS/01-Diario-individual-MiniJarvis.xlsx
+++ b/02-PROFESORADO/05-ECOSISTEMA-DIGITAL/PLANTILLAS-MAESTRAS/01-Diario-individual-MiniJarvis.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUCCIONES" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DIARIO'!$A$1:$L$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'INSTRUCCIONES'!$A$1:$B$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DIARIO'!$A$1:$G$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'INSTRUCCIONES'!$A$1:$B$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -43,7 +43,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
+        <fgColor rgb="002457A6"/>
       </patternFill>
     </fill>
   </fills>
@@ -59,13 +59,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -432,21 +429,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="19" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -457,112 +449,140 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Sesión</t>
+          <t>Hito / fase</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Hito</t>
+          <t>Objetivo o acción</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Objetivo</t>
+          <t>Prueba y resultado</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Qué hice</t>
+          <t>Enlace a evidencia</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Prueba realizada</t>
+          <t>Aprendizaje / decisión / bloqueo / siguiente paso</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>URL de evidencia</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Resultado</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Bloqueo</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Uso de IA</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Cómo validé la IA</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Siguiente paso</t>
+          <t>Uso de IA y validación (solo si procede)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Fecha de ejemplo</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>H1 · Investigar</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Comprender Scanner</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Probé entrada normal y vacía; ambas se controlan</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>URL_EJEMPLO</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Aprendí a convertir texto a número; después documentaré el caso límite</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
-      <c r="B3" s="2" t="inlineStr"/>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Fecha de ejemplo</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>H1 · Ejecutar</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Corregir conversión</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>La prueba inválida ya no cierra el programa</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>URL_EJEMPLO</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>El error fue útil; siguiente paso: añadir una prueba reproducible</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>IA para proponer casos; validé ejecutándolos</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr"/>
-      <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Fecha de ejemplo</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>H1 · Comunicar</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Preparar defensa</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Puedo ejecutar y modificar una constante</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>URL_EJEMPLO</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Necesito explicar mejor la diferencia entre variable y constante</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L4"/>
-  <dataValidations count="2">
-    <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"H0,H1,H2,H3,H4,H5,H6,H7,HF"</formula1>
-    </dataValidation>
-    <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"No,Sí"</formula1>
-    </dataValidation>
-  </dataValidations>
+  <autoFilter ref="A1:G4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -573,10 +593,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -593,55 +613,43 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Una fila por sesión o evidencia significativa</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>No convertir el diario en una narración extensa.</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Frecuencia</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>No hay fila por sesión. Registra aproximadamente investigación, ejecución y cierre, sin cuota rígida.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Enlace profundo</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Apuntar al archivo, página o commit concreto.</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Añadir entrada</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Bloqueo, decisión, error útil, IA significativa o recuperación.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>IA</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Si se usa, indicar finalidad y validación.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Privacidad</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>No introducir datos personales, credenciales ni observaciones privadas.</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Campos vacíos</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>No escribas “sin bloqueo” o “no usé IA”; deja vacío.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B5"/>
+  <autoFilter ref="A1:B4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>